<commit_message>
Updates in valuet set display bb86f1fd04d8cf62325ddc99437bf70dfd5d1d26
</commit_message>
<xml_diff>
--- a/feature/new-ig-template/ig/ValueSet-categorie-orientation-sas-valueset.xlsx
+++ b/feature/new-ig-template/ig/ValueSet-categorie-orientation-sas-valueset.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="38">
   <si>
     <t>Property</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-12T14:51:06+00:00</t>
+    <t>2026-06-15T12:26:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -121,19 +121,10 @@
     <t>604</t>
   </si>
   <si>
-    <t>CPTS</t>
-  </si>
-  <si>
     <t>603</t>
   </si>
   <si>
-    <t>MSP</t>
-  </si>
-  <si>
     <t>124</t>
-  </si>
-  <si>
-    <t>CDS</t>
   </si>
   <si>
     <t>https://mos.esante.gouv.fr/NOS/TRE_R66-CategorieEtablissement/FHIR/TRE-R66-CategorieEtablissement</t>
@@ -459,25 +450,19 @@
       <c r="A2" t="s" s="2">
         <v>34</v>
       </c>
-      <c r="B2" t="s" s="2">
-        <v>35</v>
-      </c>
+      <c r="B2" s="2"/>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
-        <v>36</v>
-      </c>
-      <c r="B3" t="s" s="2">
-        <v>37</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="B3" s="2"/>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="B4" t="s" s="2">
-        <v>39</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="B4" s="2"/>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
@@ -492,7 +477,7 @@
         <v>31</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>